<commit_message>
fix: 잔액 1,035,127 반영
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/finance/data/TO Score.xlsx
+++ b/finance/data/TO Score.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="입금현황" sheetId="1" state="visible" r:id="rId1"/>
@@ -824,14 +824,14 @@
     <cellStyle name="표준" xfId="0" builtinId="0"/>
     <cellStyle name="표준 2" xfId="1"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -842,6 +842,26 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2038,7 +2058,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W86"/>
+  <dimension ref="A1:W45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="9.375" bestFit="1" customWidth="1" style="97" min="2" max="2"/>
@@ -3623,20 +3643,20 @@
       <c r="G38" s="103" t="n"/>
       <c r="H38" s="103" t="n"/>
       <c r="I38" s="103" t="n"/>
-      <c r="J38" s="25" t="n"/>
-      <c r="K38" s="25" t="n"/>
-      <c r="L38" s="25" t="n"/>
-      <c r="M38" s="25" t="n"/>
-      <c r="N38" s="25" t="n"/>
-      <c r="O38" s="25" t="n"/>
-      <c r="P38" s="25" t="n"/>
-      <c r="Q38" s="25" t="n"/>
-      <c r="R38" s="25" t="n"/>
-      <c r="S38" s="25" t="n"/>
-      <c r="T38" s="25" t="n"/>
-      <c r="U38" s="25" t="n"/>
-      <c r="V38" s="25" t="n"/>
-      <c r="W38" s="25" t="n"/>
+      <c r="J38" s="103" t="n"/>
+      <c r="K38" s="103" t="n"/>
+      <c r="L38" s="103" t="n"/>
+      <c r="M38" s="103" t="n"/>
+      <c r="N38" s="103" t="n"/>
+      <c r="O38" s="103" t="n"/>
+      <c r="P38" s="103" t="n"/>
+      <c r="Q38" s="103" t="n"/>
+      <c r="R38" s="103" t="n"/>
+      <c r="S38" s="103" t="n"/>
+      <c r="T38" s="103" t="n"/>
+      <c r="U38" s="103" t="n"/>
+      <c r="V38" s="103" t="n"/>
+      <c r="W38" s="103" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -3663,20 +3683,20 @@
       <c r="G39" s="103" t="n"/>
       <c r="H39" s="103" t="n"/>
       <c r="I39" s="103" t="n"/>
-      <c r="J39" s="25" t="n"/>
-      <c r="K39" s="25" t="n"/>
-      <c r="L39" s="25" t="n"/>
-      <c r="M39" s="25" t="n"/>
-      <c r="N39" s="25" t="n"/>
-      <c r="O39" s="25" t="n"/>
-      <c r="P39" s="25" t="n"/>
-      <c r="Q39" s="25" t="n"/>
-      <c r="R39" s="25" t="n"/>
-      <c r="S39" s="25" t="n"/>
-      <c r="T39" s="25" t="n"/>
-      <c r="U39" s="25" t="n"/>
-      <c r="V39" s="25" t="n"/>
-      <c r="W39" s="25" t="n"/>
+      <c r="J39" s="103" t="n"/>
+      <c r="K39" s="103" t="n"/>
+      <c r="L39" s="103" t="n"/>
+      <c r="M39" s="103" t="n"/>
+      <c r="N39" s="103" t="n"/>
+      <c r="O39" s="103" t="n"/>
+      <c r="P39" s="103" t="n"/>
+      <c r="Q39" s="103" t="n"/>
+      <c r="R39" s="103" t="n"/>
+      <c r="S39" s="103" t="n"/>
+      <c r="T39" s="103" t="n"/>
+      <c r="U39" s="103" t="n"/>
+      <c r="V39" s="103" t="n"/>
+      <c r="W39" s="103" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -3953,50 +3973,14 @@
         <v/>
       </c>
     </row>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
   </sheetData>
   <conditionalFormatting sqref="A2:A43">
-    <cfRule type="duplicateValues" priority="1" dxfId="1"/>
+    <cfRule type="duplicateValues" priority="2" dxfId="0"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:W43">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
+      <formula>20000</formula>
+    </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4370,7 +4354,7 @@
         </is>
       </c>
       <c r="J16" s="118" t="n">
-        <v>1015127</v>
+        <v>1035127</v>
       </c>
     </row>
     <row r="17" ht="22.5" customHeight="1" s="97">
@@ -4428,7 +4412,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="J17">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>